<commit_message>
xlstream-eval: add skew/kurt conformance test
Register SKEW, SKEW.P, KURT in RANGE_EXPANDING_FUNCTIONS so the
classifier allows bounded range arguments.
</commit_message>
<xml_diff>
--- a/crates/xlstream-eval/tests/fixtures/statistical/skew_kurt.xlsx
+++ b/crates/xlstream-eval/tests/fixtures/statistical/skew_kurt.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t xml:space="preserve">Symmetric</t>
   </si>
@@ -38,7 +38,7 @@
     <t xml:space="preserve">Mixed</t>
   </si>
   <si>
-    <t xml:space="preserve">Error</t>
+    <t xml:space="preserve">WithErr</t>
   </si>
   <si>
     <t xml:space="preserve">Small</t>
@@ -54,6 +54,9 @@
   </si>
   <si>
     <t xml:space="preserve">text</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bool</t>
   </si>
   <si>
     <t xml:space="preserve">XS</t>
@@ -132,11 +135,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
+  <cellXfs count="1">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -417,9 +416,8 @@
       <c r="E3" s="0" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="0" t="e">
-        <f aca="false">NA()</f>
-        <v>#N/A</v>
+      <c r="F3" s="0" t="n">
+        <v>3</v>
       </c>
       <c r="G3" s="0" t="n">
         <v>20</v>
@@ -452,7 +450,7 @@
         <v>3</v>
       </c>
       <c r="F4" s="0" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G4" s="0" t="n">
         <v>30</v>
@@ -478,12 +476,8 @@
       <c r="D5" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="E5" s="1" t="b">
-        <f aca="false">TRUE()</f>
-        <v>1</v>
-      </c>
-      <c r="F5" s="0" t="n">
-        <v>5</v>
+      <c r="E5" s="0" t="s">
+        <v>11</v>
       </c>
       <c r="I5" s="0" t="n">
         <v>8</v>
@@ -592,24 +586,24 @@
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="J16" s="0" t="n">
         <f aca="false">SKEW(E2:E7)</f>
-        <v>0.541387050951085</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="J17" s="0" t="n">
         <f aca="false">KURT(E2:E7)</f>
-        <v>-1.4878892733564</v>
+        <v>-1.2</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="J18" s="0" t="e">
-        <f aca="false">SKEW(F2:F5)</f>
+        <f aca="false">SKEW(1, NA(), 3, 5)</f>
         <v>#N/A</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="J19" s="0" t="e">
-        <f aca="false">KURT(F2:F5)</f>
+        <f aca="false">KURT(1, NA(), 3, 5, 7)</f>
         <v>#N/A</v>
       </c>
     </row>
@@ -664,7 +658,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>